<commit_message>
Fix failed test case
</commit_message>
<xml_diff>
--- a/src/main/resources/testData/custDetails.xlsx
+++ b/src/main/resources/testData/custDetails.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\IdeaProjects\Selenium_Framework\src\main\resources\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\IdeaProjects\saucedemo-selenium-framework\src\main\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77552175-FE8D-4E90-9E5D-014F91861FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{879AE344-6ECE-4D4C-9266-3B377A67B9DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>First Name</t>
   </si>
@@ -40,6 +40,12 @@
   </si>
   <si>
     <t>Shinde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">John </t>
+  </si>
+  <si>
+    <t>Doe</t>
   </si>
 </sst>
 </file>
@@ -357,8 +363,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -380,6 +391,17 @@
       </c>
       <c r="C2">
         <v>411057</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3">
+        <v>415523</v>
       </c>
     </row>
   </sheetData>

</xml_diff>